<commit_message>
optimize putting matches early in the day, use cp-sat with 4 processes by default
</commit_message>
<xml_diff>
--- a/Junnutavling entries 2.xlsx
+++ b/Junnutavling entries 2.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-5020" yWindow="-19000" windowWidth="27640" windowHeight="16200" tabRatio="600" firstSheet="0" activeTab="8" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="38700" yWindow="7080" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="3" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Junnutavling entries 2" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,7 +14,8 @@
     <sheet name="Rule Violations" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="timetable_1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="timetable_2" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="timetable" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="t" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="timetable" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -40,7 +41,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="54">
     <fill>
       <patternFill/>
     </fill>
@@ -205,8 +206,80 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3E5F5"/>
-        <bgColor rgb="00F3E5F5"/>
+        <fgColor rgb="FFF3E5F5"/>
+        <bgColor rgb="FFF3E5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD1C4E9"/>
+        <bgColor rgb="FFD1C4E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1F5FE"/>
+        <bgColor rgb="FFE1F5FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB3E5FC"/>
+        <bgColor rgb="FFB3E5FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1BEE7"/>
+        <bgColor rgb="FFE1BEE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC8E6C9"/>
+        <bgColor rgb="FFC8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3F2FD"/>
+        <bgColor rgb="FFE3F2FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF81D4FA"/>
+        <bgColor rgb="FF81D4FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBBDEFB"/>
+        <bgColor rgb="FFBBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4FC3F7"/>
+        <bgColor rgb="FF4FC3F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90CAF9"/>
+        <bgColor rgb="FF90CAF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5D6A7"/>
+        <bgColor rgb="FFA5D6A7"/>
       </patternFill>
     </fill>
     <fill>
@@ -217,14 +290,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E1F5FE"/>
-        <bgColor rgb="00E1F5FE"/>
+        <fgColor rgb="00B3E5FC"/>
+        <bgColor rgb="00B3E5FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B3E5FC"/>
-        <bgColor rgb="00B3E5FC"/>
+        <fgColor rgb="004FC3F7"/>
+        <bgColor rgb="004FC3F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -235,14 +308,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E1BEE7"/>
         <bgColor rgb="00E1BEE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
-        <bgColor rgb="00C8E6C9"/>
+        <fgColor rgb="0090CAF9"/>
+        <bgColor rgb="0090CAF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1F5FE"/>
+        <bgColor rgb="00E1F5FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
+        <bgColor rgb="00F3E5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -253,32 +350,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0081D4FA"/>
-        <bgColor rgb="0081D4FA"/>
+        <fgColor rgb="00A5D6A7"/>
+        <bgColor rgb="00A5D6A7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BBDEFB"/>
-        <bgColor rgb="00BBDEFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004FC3F7"/>
-        <bgColor rgb="004FC3F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0090CAF9"/>
-        <bgColor rgb="0090CAF9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A5D6A7"/>
-        <bgColor rgb="00A5D6A7"/>
+        <fgColor rgb="0081D4FA"/>
+        <bgColor rgb="0081D4FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -294,7 +373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -327,7 +406,6 @@
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -341,6 +419,19 @@
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="49" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="50" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="43" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="53" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="46" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -739,11 +830,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D509"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col width="25.5" bestFit="1" customWidth="1" style="30" min="1" max="1"/>
-    <col width="22.83203125" bestFit="1" customWidth="1" style="30" min="3" max="3"/>
-    <col width="32.33203125" bestFit="1" customWidth="1" style="30" min="4" max="4"/>
+    <col width="25.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="22.875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="32.375" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5969,6 +6060,1077 @@
       <c r="D509" s="1" t="inlineStr">
         <is>
           <t>XD U17 Niilo Saksela (9701)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AX13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="43" t="inlineStr">
+        <is>
+          <t>GS U11 - 1</t>
+        </is>
+      </c>
+      <c r="D2" s="44" t="inlineStr">
+        <is>
+          <t>BD U11 - 1</t>
+        </is>
+      </c>
+      <c r="F2" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H2" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 1</t>
+        </is>
+      </c>
+      <c r="J2" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L2" s="44" t="inlineStr">
+        <is>
+          <t>BD U11 - 2</t>
+        </is>
+      </c>
+      <c r="N2" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="O2" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 3</t>
+        </is>
+      </c>
+      <c r="P2" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 2</t>
+        </is>
+      </c>
+      <c r="Q2" s="43" t="inlineStr">
+        <is>
+          <t>GS U11 - 3</t>
+        </is>
+      </c>
+      <c r="R2" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 3</t>
+        </is>
+      </c>
+      <c r="T2" s="44" t="inlineStr">
+        <is>
+          <t>BD U11 - 3</t>
+        </is>
+      </c>
+      <c r="V2" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 3</t>
+        </is>
+      </c>
+      <c r="W2" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 4</t>
+        </is>
+      </c>
+      <c r="X2" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 3</t>
+        </is>
+      </c>
+      <c r="Z2" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 4</t>
+        </is>
+      </c>
+      <c r="AB2" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 4</t>
+        </is>
+      </c>
+      <c r="AD2" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 4</t>
+        </is>
+      </c>
+      <c r="AF2" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 4</t>
+        </is>
+      </c>
+      <c r="AH2" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 4</t>
+        </is>
+      </c>
+      <c r="AJ2" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 5</t>
+        </is>
+      </c>
+      <c r="AL2" s="51" t="inlineStr">
+        <is>
+          <t>XD U13 - 2</t>
+        </is>
+      </c>
+      <c r="AN2" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 5</t>
+        </is>
+      </c>
+      <c r="AP2" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 5</t>
+        </is>
+      </c>
+      <c r="AT2" s="51" t="inlineStr">
+        <is>
+          <t>XD U13 - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 1</t>
+        </is>
+      </c>
+      <c r="D3" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F3" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H3" s="43" t="inlineStr">
+        <is>
+          <t>GS U11 - 2</t>
+        </is>
+      </c>
+      <c r="J3" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L3" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N3" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P3" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 2</t>
+        </is>
+      </c>
+      <c r="R3" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 3</t>
+        </is>
+      </c>
+      <c r="T3" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V3" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 3</t>
+        </is>
+      </c>
+      <c r="W3" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 4</t>
+        </is>
+      </c>
+      <c r="X3" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 3</t>
+        </is>
+      </c>
+      <c r="Z3" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 4</t>
+        </is>
+      </c>
+      <c r="AB3" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 4</t>
+        </is>
+      </c>
+      <c r="AD3" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 4</t>
+        </is>
+      </c>
+      <c r="AH3" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 4</t>
+        </is>
+      </c>
+      <c r="AL3" s="51" t="inlineStr">
+        <is>
+          <t>XD U13 - 2</t>
+        </is>
+      </c>
+      <c r="AP3" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 5</t>
+        </is>
+      </c>
+      <c r="AT3" s="51" t="inlineStr">
+        <is>
+          <t>XD U13 - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H4" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 2</t>
+        </is>
+      </c>
+      <c r="J4" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L4" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N4" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P4" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 2</t>
+        </is>
+      </c>
+      <c r="R4" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T4" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V4" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 3</t>
+        </is>
+      </c>
+      <c r="X4" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 3</t>
+        </is>
+      </c>
+      <c r="Z4" s="53" t="inlineStr">
+        <is>
+          <t>GD U15 - 3</t>
+        </is>
+      </c>
+      <c r="AD4" s="51" t="inlineStr">
+        <is>
+          <t>XD U13 - 1</t>
+        </is>
+      </c>
+      <c r="AH4" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 1</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 2</t>
+        </is>
+      </c>
+      <c r="J5" s="47" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L5" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N5" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="46" t="inlineStr">
+        <is>
+          <t>BS U11 - 2</t>
+        </is>
+      </c>
+      <c r="R5" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T5" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V5" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 3</t>
+        </is>
+      </c>
+      <c r="X5" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 3</t>
+        </is>
+      </c>
+      <c r="Z5" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 3</t>
+        </is>
+      </c>
+      <c r="AD5" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 4</t>
+        </is>
+      </c>
+      <c r="AH5" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H6" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 2</t>
+        </is>
+      </c>
+      <c r="J6" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N6" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P6" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 3</t>
+        </is>
+      </c>
+      <c r="R6" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T6" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V6" s="54" t="inlineStr">
+        <is>
+          <t>XD U17 - 3</t>
+        </is>
+      </c>
+      <c r="Z6" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D7" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>GS U13 - 2</t>
+        </is>
+      </c>
+      <c r="J7" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L7" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N7" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P7" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 3</t>
+        </is>
+      </c>
+      <c r="R7" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T7" s="53" t="inlineStr">
+        <is>
+          <t>GD U15 - 2</t>
+        </is>
+      </c>
+      <c r="V7" s="55" t="inlineStr">
+        <is>
+          <t>BD U17 - 3</t>
+        </is>
+      </c>
+      <c r="Z7" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D8" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H8" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 2</t>
+        </is>
+      </c>
+      <c r="J8" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L8" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N8" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P8" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 3</t>
+        </is>
+      </c>
+      <c r="R8" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T8" s="53" t="inlineStr">
+        <is>
+          <t>GD U15 - 2</t>
+        </is>
+      </c>
+      <c r="Z8" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D9" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H9" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 2</t>
+        </is>
+      </c>
+      <c r="J9" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L9" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N9" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P9" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R9" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H10" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 2</t>
+        </is>
+      </c>
+      <c r="J10" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L10" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N10" s="54" t="inlineStr">
+        <is>
+          <t>XD U17 - 2</t>
+        </is>
+      </c>
+      <c r="P10" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R10" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D11" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H11" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 2</t>
+        </is>
+      </c>
+      <c r="J11" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L11" s="53" t="inlineStr">
+        <is>
+          <t>GD U15 - 1</t>
+        </is>
+      </c>
+      <c r="N11" s="55" t="inlineStr">
+        <is>
+          <t>BD U17 - 2</t>
+        </is>
+      </c>
+      <c r="P11" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R11" s="52" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="50" t="inlineStr">
+        <is>
+          <t>GS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D12" s="49" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F12" s="45" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H12" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 1</t>
+        </is>
+      </c>
+      <c r="J12" s="54" t="inlineStr">
+        <is>
+          <t>GS U17 - 2</t>
+        </is>
+      </c>
+      <c r="L12" s="53" t="inlineStr">
+        <is>
+          <t>GD U15 - 1</t>
+        </is>
+      </c>
+      <c r="N12" s="55" t="inlineStr">
+        <is>
+          <t>BD U17 - 2</t>
+        </is>
+      </c>
+      <c r="P12" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R12" s="54" t="inlineStr">
+        <is>
+          <t>GS U17 - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="54" t="inlineStr">
+        <is>
+          <t>GS U17 - 1</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>BD U17 - 1</t>
+        </is>
+      </c>
+      <c r="F13" s="54" t="inlineStr">
+        <is>
+          <t>XD U17 - 1</t>
+        </is>
+      </c>
+      <c r="H13" s="50" t="inlineStr">
+        <is>
+          <t>BD U15 - 1</t>
         </is>
       </c>
     </row>
@@ -5984,7 +7146,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -6138,10 +7300,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C120"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <cols>
-    <col width="20.83203125" bestFit="1" customWidth="1" style="30" min="2" max="2"/>
-    <col width="37.6640625" bestFit="1" customWidth="1" style="30" min="3" max="3"/>
+    <col width="20.875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="37.625" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7621,10 +8783,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <cols>
-    <col width="58.1640625" bestFit="1" customWidth="1" style="30" min="2" max="2"/>
-    <col width="9.33203125" bestFit="1" customWidth="1" style="30" min="18" max="18"/>
+    <col width="58.125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.375" bestFit="1" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8504,7 +9666,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="C5:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="5">
       <c r="C5" t="inlineStr">
@@ -8561,7 +9723,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8613,7 +9775,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AX13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -9634,7 +10796,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AX13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -10640,7 +11802,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AX13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -10893,144 +12055,129 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="33" t="inlineStr">
+        <is>
+          <t>GS U11 - 1</t>
+        </is>
+      </c>
+      <c r="D2" s="32" t="inlineStr">
+        <is>
+          <t>BD U11 - 1</t>
+        </is>
+      </c>
+      <c r="F2" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H2" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 1</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 1</t>
-        </is>
-      </c>
-      <c r="F2" s="33" t="inlineStr">
-        <is>
-          <t>BD U11 - 1</t>
-        </is>
-      </c>
-      <c r="H2" s="34" t="inlineStr">
-        <is>
-          <t>GS U11 - 2</t>
-        </is>
-      </c>
-      <c r="I2" s="41" t="inlineStr">
-        <is>
-          <t>BD U17 - 1</t>
-        </is>
-      </c>
-      <c r="J2" s="31" t="inlineStr">
+      <c r="J2" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L2" s="32" t="inlineStr">
+        <is>
+          <t>BD U11 - 2</t>
+        </is>
+      </c>
+      <c r="N2" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="O2" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 3</t>
+        </is>
+      </c>
+      <c r="P2" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 2</t>
         </is>
       </c>
-      <c r="L2" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 2</t>
-        </is>
-      </c>
-      <c r="N2" s="34" t="inlineStr">
+      <c r="Q2" s="33" t="inlineStr">
         <is>
           <t>GS U11 - 3</t>
         </is>
       </c>
-      <c r="O2" s="41" t="inlineStr">
-        <is>
-          <t>BD U17 - 2</t>
-        </is>
-      </c>
-      <c r="P2" s="39" t="inlineStr">
-        <is>
-          <t>BD U13 - 2</t>
-        </is>
-      </c>
-      <c r="R2" s="31" t="inlineStr">
+      <c r="R2" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 3</t>
+        </is>
+      </c>
+      <c r="T2" s="32" t="inlineStr">
+        <is>
+          <t>BD U11 - 3</t>
+        </is>
+      </c>
+      <c r="V2" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 3</t>
+        </is>
+      </c>
+      <c r="W2" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 4</t>
+        </is>
+      </c>
+      <c r="X2" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 3</t>
         </is>
       </c>
-      <c r="T2" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 3</t>
-        </is>
-      </c>
-      <c r="V2" s="33" t="inlineStr">
-        <is>
-          <t>BD U11 - 3</t>
-        </is>
-      </c>
-      <c r="X2" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 4</t>
-        </is>
-      </c>
-      <c r="Z2" s="31" t="inlineStr">
+      <c r="Z2" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 4</t>
+        </is>
+      </c>
+      <c r="AB2" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 4</t>
+        </is>
+      </c>
+      <c r="AD2" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 4</t>
         </is>
       </c>
-      <c r="AB2" s="36" t="inlineStr">
-        <is>
-          <t>XD U13 - 1</t>
-        </is>
-      </c>
-      <c r="AD2" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 4</t>
-        </is>
-      </c>
       <c r="AF2" s="39" t="inlineStr">
         <is>
-          <t>BD U13 - 4</t>
-        </is>
-      </c>
-      <c r="AG2" s="43" t="inlineStr">
-        <is>
-          <t>GD U15 - 1</t>
-        </is>
-      </c>
-      <c r="AH2" s="40" t="inlineStr">
-        <is>
           <t>BD U15 - 4</t>
         </is>
       </c>
-      <c r="AJ2" s="36" t="inlineStr">
+      <c r="AH2" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 4</t>
+        </is>
+      </c>
+      <c r="AJ2" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 5</t>
+        </is>
+      </c>
+      <c r="AL2" s="35" t="inlineStr">
         <is>
           <t>XD U13 - 2</t>
         </is>
       </c>
-      <c r="AL2" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 5</t>
-        </is>
-      </c>
-      <c r="AM2" s="43" t="inlineStr">
-        <is>
-          <t>GD U15 - 2</t>
-        </is>
-      </c>
-      <c r="AN2" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 4</t>
-        </is>
-      </c>
-      <c r="AP2" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 4</t>
-        </is>
-      </c>
-      <c r="AR2" s="36" t="inlineStr">
+      <c r="AN2" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 5</t>
+        </is>
+      </c>
+      <c r="AP2" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 5</t>
+        </is>
+      </c>
+      <c r="AT2" s="35" t="inlineStr">
         <is>
           <t>XD U13 - 3</t>
-        </is>
-      </c>
-      <c r="AU2" s="43" t="inlineStr">
-        <is>
-          <t>GD U15 - 3</t>
-        </is>
-      </c>
-      <c r="AV2" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 5</t>
         </is>
       </c>
     </row>
@@ -11038,129 +12185,104 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="34" t="inlineStr">
-        <is>
-          <t>GS U11 - 1</t>
+      <c r="B3" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 1</t>
         </is>
       </c>
       <c r="D3" s="37" t="inlineStr">
         <is>
-          <t>GS U13 - 1</t>
-        </is>
-      </c>
-      <c r="F3" s="38" t="inlineStr">
-        <is>
           <t>BS U15 - 1</t>
         </is>
       </c>
-      <c r="H3" s="39" t="inlineStr">
-        <is>
-          <t>BD U13 - 1</t>
-        </is>
-      </c>
-      <c r="J3" s="31" t="inlineStr">
+      <c r="F3" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 1</t>
+        </is>
+      </c>
+      <c r="H3" s="33" t="inlineStr">
+        <is>
+          <t>GS U11 - 2</t>
+        </is>
+      </c>
+      <c r="J3" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L3" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N3" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P3" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 2</t>
         </is>
       </c>
-      <c r="L3" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 2</t>
-        </is>
-      </c>
-      <c r="N3" s="33" t="inlineStr">
-        <is>
-          <t>BD U11 - 2</t>
-        </is>
-      </c>
-      <c r="O3" s="41" t="inlineStr">
-        <is>
-          <t>BD U17 - 2</t>
-        </is>
-      </c>
-      <c r="P3" s="39" t="inlineStr">
-        <is>
-          <t>BD U13 - 2</t>
-        </is>
-      </c>
-      <c r="R3" s="31" t="inlineStr">
+      <c r="R3" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 3</t>
+        </is>
+      </c>
+      <c r="T3" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V3" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 3</t>
+        </is>
+      </c>
+      <c r="W3" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 4</t>
+        </is>
+      </c>
+      <c r="X3" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 3</t>
         </is>
       </c>
-      <c r="T3" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 3</t>
-        </is>
-      </c>
-      <c r="V3" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 3</t>
-        </is>
-      </c>
-      <c r="X3" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 4</t>
-        </is>
-      </c>
-      <c r="Z3" s="31" t="inlineStr">
+      <c r="Z3" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 4</t>
+        </is>
+      </c>
+      <c r="AB3" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 4</t>
+        </is>
+      </c>
+      <c r="AD3" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 4</t>
         </is>
       </c>
-      <c r="AB3" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 2</t>
-        </is>
-      </c>
-      <c r="AD3" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 4</t>
-        </is>
-      </c>
-      <c r="AF3" s="39" t="inlineStr">
-        <is>
-          <t>BD U13 - 4</t>
-        </is>
-      </c>
-      <c r="AG3" s="43" t="inlineStr">
-        <is>
-          <t>GD U15 - 1</t>
-        </is>
-      </c>
-      <c r="AH3" s="35" t="inlineStr">
-        <is>
-          <t>GS U17 - 2</t>
-        </is>
-      </c>
-      <c r="AJ3" s="36" t="inlineStr">
+      <c r="AH3" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 4</t>
+        </is>
+      </c>
+      <c r="AL3" s="35" t="inlineStr">
         <is>
           <t>XD U13 - 2</t>
         </is>
       </c>
-      <c r="AM3" s="43" t="inlineStr">
-        <is>
-          <t>GD U15 - 2</t>
-        </is>
-      </c>
-      <c r="AN3" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 4</t>
-        </is>
-      </c>
-      <c r="AP3" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 4</t>
-        </is>
-      </c>
-      <c r="AR3" s="36" t="inlineStr">
+      <c r="AP3" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 5</t>
+        </is>
+      </c>
+      <c r="AT3" s="35" t="inlineStr">
         <is>
           <t>XD U13 - 3</t>
-        </is>
-      </c>
-      <c r="AV3" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 5</t>
         </is>
       </c>
     </row>
@@ -11168,89 +12290,79 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D4" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 1</t>
-        </is>
-      </c>
-      <c r="F4" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="H4" s="35" t="inlineStr">
-        <is>
-          <t>XD U17 - 1</t>
-        </is>
-      </c>
-      <c r="J4" s="31" t="inlineStr">
+      <c r="H4" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 2</t>
+        </is>
+      </c>
+      <c r="J4" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L4" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N4" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P4" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 2</t>
         </is>
       </c>
-      <c r="L4" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 2</t>
-        </is>
-      </c>
-      <c r="N4" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="P4" s="39" t="inlineStr">
-        <is>
-          <t>BD U13 - 2</t>
-        </is>
-      </c>
-      <c r="R4" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 3</t>
-        </is>
-      </c>
-      <c r="T4" s="32" t="inlineStr">
+      <c r="R4" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T4" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V4" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 3</t>
         </is>
       </c>
-      <c r="V4" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 3</t>
-        </is>
-      </c>
       <c r="X4" s="39" t="inlineStr">
         <is>
-          <t>BD U13 - 3</t>
-        </is>
-      </c>
-      <c r="Z4" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 4</t>
-        </is>
-      </c>
-      <c r="AB4" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 2</t>
-        </is>
-      </c>
-      <c r="AJ4" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 3</t>
-        </is>
-      </c>
-      <c r="AN4" s="35" t="inlineStr">
-        <is>
-          <t>GS U17 - 3</t>
-        </is>
-      </c>
-      <c r="AV4" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 5</t>
+          <t>BD U15 - 3</t>
+        </is>
+      </c>
+      <c r="Z4" s="42" t="inlineStr">
+        <is>
+          <t>GD U15 - 3</t>
+        </is>
+      </c>
+      <c r="AD4" s="35" t="inlineStr">
+        <is>
+          <t>XD U13 - 1</t>
+        </is>
+      </c>
+      <c r="AH4" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 4</t>
         </is>
       </c>
     </row>
@@ -11258,74 +12370,79 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="32" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 1</t>
+        </is>
+      </c>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F5" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D5" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="F5" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
+      <c r="H5" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 2</t>
+        </is>
+      </c>
+      <c r="J5" s="38" t="inlineStr">
+        <is>
+          <t>BD U13 - 2</t>
+        </is>
+      </c>
+      <c r="L5" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N5" s="31" t="inlineStr">
+        <is>
+          <t>BS U13 - 2</t>
+        </is>
+      </c>
+      <c r="P5" s="30" t="inlineStr">
         <is>
           <t>BS U11 - 2</t>
         </is>
       </c>
-      <c r="L5" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 2</t>
-        </is>
-      </c>
-      <c r="N5" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="P5" s="39" t="inlineStr">
-        <is>
-          <t>BD U13 - 2</t>
-        </is>
-      </c>
-      <c r="R5" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 3</t>
-        </is>
-      </c>
-      <c r="T5" s="32" t="inlineStr">
+      <c r="R5" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T5" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 3</t>
+        </is>
+      </c>
+      <c r="V5" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 3</t>
         </is>
       </c>
-      <c r="V5" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 3</t>
-        </is>
-      </c>
       <c r="X5" s="39" t="inlineStr">
         <is>
-          <t>BD U13 - 3</t>
-        </is>
-      </c>
-      <c r="Z5" s="40" t="inlineStr">
-        <is>
           <t>BD U15 - 3</t>
         </is>
       </c>
-      <c r="AB5" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 2</t>
-        </is>
-      </c>
-      <c r="AJ5" s="42" t="inlineStr">
+      <c r="Z5" s="41" t="inlineStr">
         <is>
           <t>BS U17 - 3</t>
+        </is>
+      </c>
+      <c r="AD5" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 4</t>
+        </is>
+      </c>
+      <c r="AH5" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 4</t>
         </is>
       </c>
     </row>
@@ -11333,72 +12450,62 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="32" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D6" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J6" s="37" t="inlineStr">
+      <c r="H6" s="36" t="inlineStr">
         <is>
           <t>GS U13 - 2</t>
         </is>
       </c>
-      <c r="L6" s="32" t="inlineStr">
+      <c r="J6" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N6" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 2</t>
         </is>
       </c>
-      <c r="N6" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="P6" s="35" t="inlineStr">
-        <is>
-          <t>XD U17 - 2</t>
-        </is>
-      </c>
-      <c r="R6" s="40" t="inlineStr">
-        <is>
-          <t>BD U15 - 2</t>
-        </is>
-      </c>
-      <c r="T6" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 3</t>
-        </is>
-      </c>
-      <c r="V6" s="38" t="inlineStr">
+      <c r="P6" s="36" t="inlineStr">
+        <is>
+          <t>GS U13 - 3</t>
+        </is>
+      </c>
+      <c r="R6" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T6" s="37" t="inlineStr">
         <is>
           <t>BS U15 - 3</t>
         </is>
       </c>
-      <c r="X6" s="35" t="inlineStr">
+      <c r="V6" s="34" t="inlineStr">
         <is>
           <t>XD U17 - 3</t>
         </is>
       </c>
-      <c r="Z6" s="40" t="inlineStr">
-        <is>
-          <t>BD U15 - 3</t>
-        </is>
-      </c>
-      <c r="AB6" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 2</t>
-        </is>
-      </c>
-      <c r="AJ6" s="42" t="inlineStr">
+      <c r="Z6" s="41" t="inlineStr">
         <is>
           <t>BS U17 - 3</t>
         </is>
@@ -11408,57 +12515,62 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="32" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D7" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F7" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="F7" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J7" s="37" t="inlineStr">
+      <c r="H7" s="36" t="inlineStr">
         <is>
           <t>GS U13 - 2</t>
         </is>
       </c>
-      <c r="L7" s="32" t="inlineStr">
+      <c r="J7" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L7" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N7" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 2</t>
         </is>
       </c>
-      <c r="N7" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="R7" s="40" t="inlineStr">
-        <is>
-          <t>BD U15 - 2</t>
-        </is>
-      </c>
-      <c r="T7" s="40" t="inlineStr">
+      <c r="P7" s="39" t="inlineStr">
         <is>
           <t>GS U15 - 3</t>
         </is>
       </c>
-      <c r="X7" s="41" t="inlineStr">
+      <c r="R7" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
+        </is>
+      </c>
+      <c r="T7" s="42" t="inlineStr">
+        <is>
+          <t>GD U15 - 2</t>
+        </is>
+      </c>
+      <c r="V7" s="40" t="inlineStr">
         <is>
           <t>BD U17 - 3</t>
         </is>
       </c>
-      <c r="AB7" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 2</t>
-        </is>
-      </c>
-      <c r="AJ7" s="42" t="inlineStr">
+      <c r="Z7" s="41" t="inlineStr">
         <is>
           <t>BS U17 - 3</t>
         </is>
@@ -11468,49 +12580,59 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D8" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="F8" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J8" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 2</t>
-        </is>
-      </c>
-      <c r="L8" s="32" t="inlineStr">
+      <c r="H8" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 2</t>
+        </is>
+      </c>
+      <c r="J8" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L8" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N8" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 2</t>
         </is>
       </c>
-      <c r="N8" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="R8" s="40" t="inlineStr">
-        <is>
-          <t>BD U15 - 2</t>
+      <c r="P8" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 3</t>
+        </is>
+      </c>
+      <c r="R8" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
         </is>
       </c>
       <c r="T8" s="42" t="inlineStr">
         <is>
-          <t>BS U17 - 1</t>
-        </is>
-      </c>
-      <c r="AB8" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 2</t>
+          <t>GD U15 - 2</t>
+        </is>
+      </c>
+      <c r="Z8" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 3</t>
         </is>
       </c>
     </row>
@@ -11518,47 +12640,47 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="32" t="inlineStr">
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D9" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="F9" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J9" s="37" t="inlineStr">
-        <is>
-          <t>GS U13 - 2</t>
-        </is>
-      </c>
-      <c r="L9" s="32" t="inlineStr">
+      <c r="H9" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 2</t>
+        </is>
+      </c>
+      <c r="J9" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L9" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 2</t>
+        </is>
+      </c>
+      <c r="N9" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 2</t>
         </is>
       </c>
-      <c r="N9" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="R9" s="40" t="inlineStr">
+      <c r="P9" s="39" t="inlineStr">
         <is>
           <t>BD U15 - 2</t>
         </is>
       </c>
-      <c r="T9" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 1</t>
-        </is>
-      </c>
-      <c r="AB9" s="42" t="inlineStr">
+      <c r="R9" s="41" t="inlineStr">
         <is>
           <t>BS U17 - 2</t>
         </is>
@@ -11568,42 +12690,47 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D10" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="F10" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J10" s="40" t="inlineStr">
-        <is>
-          <t>BD U15 - 1</t>
-        </is>
-      </c>
-      <c r="L10" s="40" t="inlineStr">
+      <c r="H10" s="39" t="inlineStr">
         <is>
           <t>GS U15 - 2</t>
         </is>
       </c>
-      <c r="N10" s="38" t="inlineStr">
+      <c r="J10" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 1</t>
+        </is>
+      </c>
+      <c r="L10" s="37" t="inlineStr">
         <is>
           <t>BS U15 - 2</t>
         </is>
       </c>
-      <c r="T10" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 1</t>
-        </is>
-      </c>
-      <c r="AB10" s="42" t="inlineStr">
+      <c r="N10" s="34" t="inlineStr">
+        <is>
+          <t>XD U17 - 2</t>
+        </is>
+      </c>
+      <c r="P10" s="39" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R10" s="41" t="inlineStr">
         <is>
           <t>BS U17 - 2</t>
         </is>
@@ -11613,39 +12740,49 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F11" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D11" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="J11" s="40" t="inlineStr">
-        <is>
-          <t>BD U15 - 1</t>
-        </is>
-      </c>
-      <c r="L11" s="40" t="inlineStr">
+      <c r="H11" s="39" t="inlineStr">
         <is>
           <t>GS U15 - 2</t>
         </is>
       </c>
-      <c r="N11" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 2</t>
-        </is>
-      </c>
-      <c r="T11" s="42" t="inlineStr">
+      <c r="J11" s="41" t="inlineStr">
         <is>
           <t>BS U17 - 1</t>
         </is>
       </c>
-      <c r="AB11" s="35" t="inlineStr">
-        <is>
-          <t>GS U17 - 1</t>
+      <c r="L11" s="42" t="inlineStr">
+        <is>
+          <t>GD U15 - 1</t>
+        </is>
+      </c>
+      <c r="N11" s="40" t="inlineStr">
+        <is>
+          <t>BD U17 - 2</t>
+        </is>
+      </c>
+      <c r="P11" s="39" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R11" s="41" t="inlineStr">
+        <is>
+          <t>BS U17 - 2</t>
         </is>
       </c>
     </row>
@@ -11653,24 +12790,49 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
+        <is>
+          <t>GS U15 - 1</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>BS U15 - 1</t>
+        </is>
+      </c>
+      <c r="F12" s="31" t="inlineStr">
         <is>
           <t>BS U13 - 1</t>
         </is>
       </c>
-      <c r="D12" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="L12" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 2</t>
-        </is>
-      </c>
-      <c r="T12" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 1</t>
+      <c r="H12" s="39" t="inlineStr">
+        <is>
+          <t>BD U15 - 1</t>
+        </is>
+      </c>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
+          <t>GS U17 - 2</t>
+        </is>
+      </c>
+      <c r="L12" s="42" t="inlineStr">
+        <is>
+          <t>GD U15 - 1</t>
+        </is>
+      </c>
+      <c r="N12" s="40" t="inlineStr">
+        <is>
+          <t>BD U17 - 2</t>
+        </is>
+      </c>
+      <c r="P12" s="39" t="inlineStr">
+        <is>
+          <t>BD U15 - 2</t>
+        </is>
+      </c>
+      <c r="R12" s="34" t="inlineStr">
+        <is>
+          <t>GS U17 - 3</t>
         </is>
       </c>
     </row>
@@ -11678,24 +12840,24 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="32" t="inlineStr">
-        <is>
-          <t>BS U13 - 1</t>
-        </is>
-      </c>
-      <c r="D13" s="38" t="inlineStr">
-        <is>
-          <t>BS U15 - 1</t>
-        </is>
-      </c>
-      <c r="L13" s="40" t="inlineStr">
-        <is>
-          <t>GS U15 - 2</t>
-        </is>
-      </c>
-      <c r="T13" s="42" t="inlineStr">
-        <is>
-          <t>BS U17 - 1</t>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>GS U17 - 1</t>
+        </is>
+      </c>
+      <c r="D13" s="40" t="inlineStr">
+        <is>
+          <t>BD U17 - 1</t>
+        </is>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>XD U17 - 1</t>
+        </is>
+      </c>
+      <c r="H13" s="39" t="inlineStr">
+        <is>
+          <t>BD U15 - 1</t>
         </is>
       </c>
     </row>

</xml_diff>